<commit_message>
Init function separation for simpler dual core initiation
</commit_message>
<xml_diff>
--- a/Autogen/UniversalDataBlock.xlsx
+++ b/Autogen/UniversalDataBlock.xlsx
@@ -97,9 +97,6 @@
     <t xml:space="preserve">Map Gen Second</t>
   </si>
   <si>
-    <t xml:space="preserve">Map Number Of Blocks</t>
-  </si>
-  <si>
     <t xml:space="preserve">Map Checksum</t>
   </si>
   <si>
@@ -125,6 +122,9 @@
   </si>
   <si>
     <t xml:space="preserve">Watchdog Timeout</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Watchdog Counter</t>
   </si>
   <si>
     <t xml:space="preserve">Watchdog Fault Active</t>
@@ -684,7 +684,7 @@
         <v>25</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>11</v>
@@ -710,30 +710,30 @@
         <v>26</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="D11" s="1" t="s">
         <v>12</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>12</v>
+        <v>28</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="H11" s="3" t="s">
-        <v>13</v>
+        <v>29</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="B12" s="1" t="s">
         <v>19</v>
@@ -745,16 +745,16 @@
         <v>12</v>
       </c>
       <c r="E12" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="F12" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="F12" s="1" t="s">
+      <c r="G12" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="H12" s="3" t="s">
         <v>29</v>
-      </c>
-      <c r="G12" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="H12" s="3" t="s">
-        <v>30</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -771,16 +771,16 @@
         <v>12</v>
       </c>
       <c r="E13" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="F13" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="F13" s="1" t="s">
+      <c r="G13" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="H13" s="3" t="s">
         <v>29</v>
-      </c>
-      <c r="G13" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="H13" s="3" t="s">
-        <v>30</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -797,16 +797,16 @@
         <v>12</v>
       </c>
       <c r="E14" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="F14" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="F14" s="1" t="s">
+      <c r="G14" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="H14" s="3" t="s">
         <v>29</v>
-      </c>
-      <c r="G14" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="H14" s="3" t="s">
-        <v>30</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -814,7 +814,7 @@
         <v>33</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="C15" s="1" t="s">
         <v>16</v>
@@ -823,16 +823,16 @@
         <v>12</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>28</v>
+        <v>12</v>
       </c>
       <c r="F15" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="G15" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="H15" s="3" t="s">
         <v>29</v>
-      </c>
-      <c r="G15" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="H15" s="3" t="s">
-        <v>30</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -843,7 +843,7 @@
         <v>15</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="D16" s="1" t="s">
         <v>12</v>
@@ -855,10 +855,10 @@
         <v>12</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>28</v>
+        <v>12</v>
       </c>
       <c r="H16" s="3" t="s">
-        <v>30</v>
+        <v>13</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
initUniversalInfo implemented - testing required. CRC & COBs errors added to Universal Data Block.
</commit_message>
<xml_diff>
--- a/Autogen/UniversalDataBlock.xlsx
+++ b/Autogen/UniversalDataBlock.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="43">
   <si>
     <t xml:space="preserve">Member ID</t>
   </si>
@@ -131,6 +131,15 @@
   </si>
   <si>
     <t xml:space="preserve">Watchdog Reset</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CRC Error Count</t>
+  </si>
+  <si>
+    <t xml:space="preserve">uin32_t</t>
+  </si>
+  <si>
+    <t xml:space="preserve">COBS Error Count</t>
   </si>
   <si>
     <t xml:space="preserve">Store NVM</t>
@@ -428,7 +437,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I21"/>
+  <dimension ref="A1:I23"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="52.6"/>
@@ -918,10 +927,10 @@
         <v>37</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="D19" s="1" t="s">
         <v>12</v>
@@ -941,13 +950,13 @@
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B20" s="1" t="s">
         <v>15</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="D20" s="1" t="s">
         <v>12</v>
@@ -967,33 +976,85 @@
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B21" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="E21" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F21" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="G21" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="H21" s="3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="E22" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F22" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="G22" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="H22" s="3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B23" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="C21" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D21" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="E21" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="F21" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="G21" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="H21" s="3" t="s">
+      <c r="C23" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D23" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="E23" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F23" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="G23" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="H23" s="3" t="s">
         <v>13</v>
       </c>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="H2:H21" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="H2:H23" type="list">
       <formula1>"NO,YES"</formula1>
       <formula2>0</formula2>
     </dataValidation>

</xml_diff>

<commit_message>
Node init NVM extraction procedure in progress
</commit_message>
<xml_diff>
--- a/Autogen/UniversalDataBlock.xlsx
+++ b/Autogen/UniversalDataBlock.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="193" uniqueCount="42">
   <si>
     <t xml:space="preserve">Member ID</t>
   </si>
@@ -49,10 +49,10 @@
     <t xml:space="preserve">Description</t>
   </si>
   <si>
-    <t xml:space="preserve">Atams Version Number</t>
-  </si>
-  <si>
-    <t xml:space="preserve">float</t>
+    <t xml:space="preserve">Atams Version Major</t>
+  </si>
+  <si>
+    <t xml:space="preserve">uint8_t</t>
   </si>
   <si>
     <t xml:space="preserve">RO</t>
@@ -64,7 +64,10 @@
     <t xml:space="preserve">NO</t>
   </si>
   <si>
-    <t xml:space="preserve">Universal Unlock</t>
+    <t xml:space="preserve">Atams Version Minor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Universal Write Unlock</t>
   </si>
   <si>
     <t xml:space="preserve">uint32_t</t>
@@ -79,9 +82,6 @@
     <t xml:space="preserve">Map Gen Month</t>
   </si>
   <si>
-    <t xml:space="preserve">uint8_t</t>
-  </si>
-  <si>
     <t xml:space="preserve">Map Gen Year</t>
   </si>
   <si>
@@ -104,9 +104,6 @@
   </si>
   <si>
     <t xml:space="preserve">0</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NODE_ID_MAX</t>
   </si>
   <si>
     <t xml:space="preserve">YES</t>
@@ -437,7 +434,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I23"/>
+  <dimension ref="A1:I24"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="52.6"/>
@@ -511,10 +508,10 @@
         <v>14</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>12</v>
@@ -534,13 +531,13 @@
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C4" s="1" t="s">
         <v>17</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>11</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>12</v>
@@ -563,7 +560,7 @@
         <v>18</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>11</v>
@@ -586,10 +583,10 @@
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>21</v>
+        <v>10</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>11</v>
@@ -612,10 +609,10 @@
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>11</v>
@@ -638,10 +635,10 @@
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>11</v>
@@ -664,10 +661,10 @@
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="C9" s="1" t="s">
         <v>11</v>
@@ -690,10 +687,10 @@
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>11</v>
@@ -716,117 +713,117 @@
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="D11" s="1" t="s">
         <v>12</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>28</v>
+        <v>12</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="H11" s="3" t="s">
-        <v>29</v>
+        <v>13</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D12" s="1" t="s">
         <v>12</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>28</v>
+        <v>12</v>
       </c>
       <c r="G12" s="1" t="s">
         <v>27</v>
       </c>
       <c r="H12" s="3" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D13" s="1" t="s">
         <v>12</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>28</v>
+        <v>12</v>
       </c>
       <c r="G13" s="1" t="s">
         <v>27</v>
       </c>
       <c r="H13" s="3" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D14" s="1" t="s">
         <v>12</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>28</v>
+        <v>12</v>
       </c>
       <c r="G14" s="1" t="s">
         <v>27</v>
       </c>
       <c r="H14" s="3" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D15" s="1" t="s">
         <v>12</v>
@@ -841,18 +838,18 @@
         <v>27</v>
       </c>
       <c r="H15" s="3" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="D16" s="1" t="s">
         <v>12</v>
@@ -864,18 +861,18 @@
         <v>12</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="H16" s="3" t="s">
-        <v>13</v>
+        <v>28</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="C17" s="1" t="s">
         <v>11</v>
@@ -898,13 +895,13 @@
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="D18" s="1" t="s">
         <v>12</v>
@@ -924,13 +921,13 @@
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>38</v>
+        <v>10</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="D19" s="1" t="s">
         <v>12</v>
@@ -950,10 +947,10 @@
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>15</v>
+        <v>37</v>
       </c>
       <c r="C20" s="1" t="s">
         <v>11</v>
@@ -976,13 +973,13 @@
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="D21" s="1" t="s">
         <v>12</v>
@@ -1002,13 +999,13 @@
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D22" s="1" t="s">
         <v>12</v>
@@ -1028,13 +1025,13 @@
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="D23" s="1" t="s">
         <v>12</v>
@@ -1049,12 +1046,38 @@
         <v>12</v>
       </c>
       <c r="H23" s="3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D24" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="E24" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F24" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="G24" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="H24" s="3" t="s">
         <v>13</v>
       </c>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="H2:H23" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="H2:H24" type="list">
       <formula1>"NO,YES"</formula1>
       <formula2>0</formula2>
     </dataValidation>

</xml_diff>

<commit_message>
Node configuration state functionality in progress
</commit_message>
<xml_diff>
--- a/Autogen/UniversalDataBlock.xlsx
+++ b/Autogen/UniversalDataBlock.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="241" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="232" uniqueCount="47">
   <si>
     <t xml:space="preserve">Member ID</t>
   </si>
@@ -61,91 +61,94 @@
     <t xml:space="preserve">-</t>
   </si>
   <si>
+    <t xml:space="preserve">false</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Atams Version Minor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Map Gen Day</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Map Gen Month</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Map Gen Year</t>
+  </si>
+  <si>
+    <t xml:space="preserve">uint16_t</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Map Gen Hour</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Map Gen Minute</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Map Gen Second</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Map Checksum</t>
+  </si>
+  <si>
+    <t xml:space="preserve">uint32_t</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Configuration Passkey</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RW</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ACCESS_KEY, APPLY_KEY</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Configuration Status</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DENIED, APPLIED, CANCELLED</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Node ID</t>
+  </si>
+  <si>
     <t xml:space="preserve">true</t>
   </si>
   <si>
-    <t xml:space="preserve">Atams Version Minor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Map Gen Day</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Map Gen Month</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Map Gen Year</t>
-  </si>
-  <si>
-    <t xml:space="preserve">uint16_t</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Map Gen Hour</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Map Gen Minute</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Map Gen Second</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Map Checksum</t>
-  </si>
-  <si>
-    <t xml:space="preserve">uint32_t</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Universal Unlock</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RW</t>
-  </si>
-  <si>
-    <t xml:space="preserve">false</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Node ID Set</t>
-  </si>
-  <si>
-    <t xml:space="preserve">First Node ID Set</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Last Node ID Set</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Previous Node ID Set</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Node ID Display</t>
-  </si>
-  <si>
-    <t xml:space="preserve">First Node ID Display</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Last Node ID Display</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Previous Node ID Display</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Apply Identifiers</t>
+    <t xml:space="preserve">First Node ID</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Last Node ID</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Previous Node ID</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bitrate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Watchdog Period</t>
   </si>
   <si>
     <t xml:space="preserve">Store All</t>
   </si>
   <si>
+    <t xml:space="preserve">Passcode</t>
+  </si>
+  <si>
     <t xml:space="preserve">Restore User Blocks</t>
   </si>
   <si>
     <t xml:space="preserve">Restore All</t>
   </si>
   <si>
+    <t xml:space="preserve">Reset Node</t>
+  </si>
+  <si>
     <t xml:space="preserve">Storage Status</t>
   </si>
   <si>
     <t xml:space="preserve">Storage Process Complete</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Watchdog Timeout</t>
   </si>
   <si>
     <t xml:space="preserve">Watchdog Fault Active</t>
@@ -450,7 +453,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I36"/>
+  <dimension ref="A1:I39"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="52.6"/>
@@ -732,7 +735,7 @@
         <v>24</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>23</v>
+        <v>10</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>25</v>
@@ -750,6 +753,9 @@
         <v>12</v>
       </c>
       <c r="H11" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="I11" s="1" t="s">
         <v>26</v>
       </c>
     </row>
@@ -761,7 +767,7 @@
         <v>10</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>25</v>
+        <v>11</v>
       </c>
       <c r="D12" s="1" t="s">
         <v>12</v>
@@ -776,12 +782,15 @@
         <v>12</v>
       </c>
       <c r="H12" s="3" t="s">
-        <v>26</v>
+        <v>13</v>
+      </c>
+      <c r="I12" s="1" t="s">
+        <v>28</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B13" s="3" t="s">
         <v>10</v>
@@ -802,12 +811,12 @@
         <v>12</v>
       </c>
       <c r="H13" s="3" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B14" s="3" t="s">
         <v>10</v>
@@ -828,12 +837,12 @@
         <v>12</v>
       </c>
       <c r="H14" s="3" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B15" s="3" t="s">
         <v>10</v>
@@ -854,18 +863,18 @@
         <v>12</v>
       </c>
       <c r="H15" s="3" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B16" s="3" t="s">
         <v>10</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="D16" s="1" t="s">
         <v>12</v>
@@ -880,18 +889,18 @@
         <v>12</v>
       </c>
       <c r="H16" s="3" t="s">
-        <v>13</v>
+        <v>30</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B17" s="3" t="s">
         <v>10</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="D17" s="1" t="s">
         <v>12</v>
@@ -906,18 +915,18 @@
         <v>12</v>
       </c>
       <c r="H17" s="3" t="s">
-        <v>13</v>
+        <v>30</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>10</v>
+        <v>23</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="D18" s="1" t="s">
         <v>12</v>
@@ -932,18 +941,18 @@
         <v>12</v>
       </c>
       <c r="H18" s="3" t="s">
-        <v>13</v>
+        <v>30</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>10</v>
+        <v>23</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="D19" s="1" t="s">
         <v>12</v>
@@ -959,11 +968,14 @@
       </c>
       <c r="H19" s="3" t="s">
         <v>13</v>
+      </c>
+      <c r="I19" s="1" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="B20" s="3" t="s">
         <v>23</v>
@@ -984,12 +996,15 @@
         <v>12</v>
       </c>
       <c r="H20" s="3" t="s">
-        <v>26</v>
+        <v>13</v>
+      </c>
+      <c r="I20" s="1" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="B21" s="3" t="s">
         <v>23</v>
@@ -1010,12 +1025,15 @@
         <v>12</v>
       </c>
       <c r="H21" s="3" t="s">
-        <v>26</v>
+        <v>13</v>
+      </c>
+      <c r="I21" s="1" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="B22" s="3" t="s">
         <v>23</v>
@@ -1036,18 +1054,21 @@
         <v>12</v>
       </c>
       <c r="H22" s="3" t="s">
-        <v>26</v>
+        <v>13</v>
+      </c>
+      <c r="I22" s="1" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>23</v>
+        <v>10</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>25</v>
+        <v>11</v>
       </c>
       <c r="D23" s="1" t="s">
         <v>12</v>
@@ -1062,12 +1083,12 @@
         <v>12</v>
       </c>
       <c r="H23" s="3" t="s">
-        <v>26</v>
+        <v>13</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="B24" s="3" t="s">
         <v>10</v>
@@ -1087,13 +1108,13 @@
       <c r="G24" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="H24" s="3" t="s">
-        <v>26</v>
+      <c r="H24" s="1" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="1" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="B25" s="3" t="s">
         <v>10</v>
@@ -1113,13 +1134,13 @@
       <c r="G25" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="H25" s="1" t="s">
-        <v>26</v>
+      <c r="H25" s="3" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="B26" s="3" t="s">
         <v>23</v>
@@ -1142,13 +1163,16 @@
       <c r="H26" s="3" t="s">
         <v>13</v>
       </c>
+      <c r="I26" s="1" t="s">
+        <v>37</v>
+      </c>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="1" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>10</v>
+        <v>23</v>
       </c>
       <c r="C27" s="1" t="s">
         <v>11</v>
@@ -1166,18 +1190,18 @@
         <v>12</v>
       </c>
       <c r="H27" s="3" t="s">
-        <v>26</v>
+        <v>13</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="1" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>10</v>
+        <v>23</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>25</v>
+        <v>11</v>
       </c>
       <c r="D28" s="1" t="s">
         <v>12</v>
@@ -1192,60 +1216,58 @@
         <v>12</v>
       </c>
       <c r="H28" s="3" t="s">
-        <v>26</v>
+        <v>13</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="B29" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="C29" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D29" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="E29" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="F29" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="G29" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="H29" s="3" t="s">
-        <v>26</v>
-      </c>
+      <c r="A29" s="4"/>
+      <c r="B29" s="4"/>
+      <c r="C29" s="4"/>
+      <c r="D29" s="4"/>
+      <c r="E29" s="4"/>
+      <c r="F29" s="4"/>
+      <c r="G29" s="4"/>
+      <c r="H29" s="4"/>
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="B30" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="C30" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D30" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="E30" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="F30" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="G30" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="H30" s="3" t="s">
-        <v>26</v>
-      </c>
+      <c r="A30" s="4"/>
+      <c r="B30" s="4"/>
+      <c r="C30" s="4"/>
+      <c r="D30" s="4"/>
+      <c r="E30" s="4"/>
+      <c r="F30" s="4"/>
+      <c r="G30" s="4"/>
+      <c r="H30" s="4"/>
+    </row>
+    <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="4"/>
+      <c r="B31" s="4"/>
+      <c r="C31" s="4"/>
+      <c r="D31" s="4"/>
+      <c r="E31" s="4"/>
+      <c r="F31" s="4"/>
+      <c r="G31" s="4"/>
+      <c r="H31" s="4"/>
+    </row>
+    <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="4"/>
+      <c r="B32" s="4"/>
+      <c r="C32" s="4"/>
+      <c r="D32" s="4"/>
+      <c r="E32" s="4"/>
+      <c r="F32" s="4"/>
+      <c r="G32" s="4"/>
+      <c r="H32" s="4"/>
+    </row>
+    <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="4"/>
+      <c r="B33" s="4"/>
+      <c r="C33" s="4"/>
+      <c r="D33" s="4"/>
+      <c r="E33" s="4"/>
+      <c r="F33" s="4"/>
+      <c r="G33" s="4"/>
+      <c r="H33" s="4"/>
     </row>
     <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="4"/>
@@ -1257,33 +1279,33 @@
       <c r="G34" s="4"/>
       <c r="H34" s="4"/>
     </row>
-    <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="4"/>
-      <c r="B35" s="4"/>
-      <c r="C35" s="4"/>
-      <c r="D35" s="4"/>
-      <c r="E35" s="4"/>
-      <c r="F35" s="4"/>
-      <c r="G35" s="4"/>
-      <c r="H35" s="4"/>
-    </row>
-    <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="4"/>
-      <c r="B36" s="4"/>
-      <c r="C36" s="4"/>
-      <c r="D36" s="4"/>
-      <c r="E36" s="4"/>
-      <c r="F36" s="4"/>
-      <c r="G36" s="4"/>
-      <c r="H36" s="4"/>
+    <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="4"/>
+      <c r="B38" s="4"/>
+      <c r="C38" s="4"/>
+      <c r="D38" s="4"/>
+      <c r="E38" s="4"/>
+      <c r="F38" s="4"/>
+      <c r="G38" s="4"/>
+      <c r="H38" s="4"/>
+    </row>
+    <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="4"/>
+      <c r="B39" s="4"/>
+      <c r="C39" s="4"/>
+      <c r="D39" s="4"/>
+      <c r="E39" s="4"/>
+      <c r="F39" s="4"/>
+      <c r="G39" s="4"/>
+      <c r="H39" s="4"/>
     </row>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="H2:H24 H26:H30" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="H2:H23 H25:H28" type="list">
       <formula1>"true,false"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="B2:B30" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="B2:B28" type="list">
       <formula1>"uint8_t,int8_t,uint16_t,int16_t,uint32_t,int32_t,float"</formula1>
       <formula2>0</formula2>
     </dataValidation>

</xml_diff>

<commit_message>
Node - Number of nodes added to GenInfo + RTTI requirement removal + Data Block removal from Datagram Header
</commit_message>
<xml_diff>
--- a/Autogen/UniversalDataBlock.xlsx
+++ b/Autogen/UniversalDataBlock.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="232" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="240" uniqueCount="48">
   <si>
     <t xml:space="preserve">Member ID</t>
   </si>
@@ -86,6 +86,9 @@
   </si>
   <si>
     <t xml:space="preserve">Map Gen Second</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Map Number of Vars</t>
   </si>
   <si>
     <t xml:space="preserve">Map Checksum</t>
@@ -453,7 +456,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I39"/>
+  <dimension ref="A1:I40"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="52.6"/>
@@ -709,7 +712,7 @@
         <v>22</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>11</v>
@@ -732,13 +735,13 @@
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B11" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="B11" s="3" t="s">
-        <v>10</v>
-      </c>
       <c r="C11" s="1" t="s">
-        <v>25</v>
+        <v>11</v>
       </c>
       <c r="D11" s="1" t="s">
         <v>12</v>
@@ -754,90 +757,90 @@
       </c>
       <c r="H11" s="3" t="s">
         <v>13</v>
-      </c>
-      <c r="I11" s="1" t="s">
-        <v>26</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="G12" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="H12" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="I12" s="1" t="s">
         <v>27</v>
-      </c>
-      <c r="B12" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="C12" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D12" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="E12" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="F12" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="G12" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="H12" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="I12" s="1" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F13" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="G13" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="H13" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="I13" s="1" t="s">
         <v>29</v>
-      </c>
-      <c r="B13" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="C13" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="D13" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="E13" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="F13" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="G13" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="H13" s="3" t="s">
-        <v>30</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F14" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="G14" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="H14" s="3" t="s">
         <v>31</v>
-      </c>
-      <c r="B14" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="C14" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="D14" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="E14" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="F14" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="G14" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="H14" s="3" t="s">
-        <v>30</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -848,7 +851,7 @@
         <v>10</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D15" s="1" t="s">
         <v>12</v>
@@ -863,7 +866,7 @@
         <v>12</v>
       </c>
       <c r="H15" s="3" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -874,7 +877,7 @@
         <v>10</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D16" s="1" t="s">
         <v>12</v>
@@ -889,7 +892,7 @@
         <v>12</v>
       </c>
       <c r="H16" s="3" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -900,7 +903,7 @@
         <v>10</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D17" s="1" t="s">
         <v>12</v>
@@ -915,7 +918,7 @@
         <v>12</v>
       </c>
       <c r="H17" s="3" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -923,10 +926,10 @@
         <v>35</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>23</v>
+        <v>10</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D18" s="1" t="s">
         <v>12</v>
@@ -941,7 +944,7 @@
         <v>12</v>
       </c>
       <c r="H18" s="3" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -949,10 +952,10 @@
         <v>36</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D19" s="1" t="s">
         <v>12</v>
@@ -967,39 +970,36 @@
         <v>12</v>
       </c>
       <c r="H19" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="I19" s="1" t="s">
-        <v>37</v>
+        <v>31</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F20" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="G20" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="H20" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="I20" s="1" t="s">
         <v>38</v>
-      </c>
-      <c r="B20" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="C20" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="D20" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="E20" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="F20" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="G20" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="H20" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="I20" s="1" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1007,10 +1007,10 @@
         <v>39</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D21" s="1" t="s">
         <v>12</v>
@@ -1028,7 +1028,7 @@
         <v>13</v>
       </c>
       <c r="I21" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1036,10 +1036,10 @@
         <v>40</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D22" s="1" t="s">
         <v>12</v>
@@ -1057,7 +1057,7 @@
         <v>13</v>
       </c>
       <c r="I22" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1065,10 +1065,10 @@
         <v>41</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>10</v>
+        <v>24</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="D23" s="1" t="s">
         <v>12</v>
@@ -1084,6 +1084,9 @@
       </c>
       <c r="H23" s="3" t="s">
         <v>13</v>
+      </c>
+      <c r="I23" s="1" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1108,7 +1111,7 @@
       <c r="G24" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="H24" s="1" t="s">
+      <c r="H24" s="3" t="s">
         <v>13</v>
       </c>
     </row>
@@ -1134,7 +1137,7 @@
       <c r="G25" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="H25" s="3" t="s">
+      <c r="H25" s="1" t="s">
         <v>13</v>
       </c>
     </row>
@@ -1143,10 +1146,10 @@
         <v>44</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>23</v>
+        <v>10</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>25</v>
+        <v>11</v>
       </c>
       <c r="D26" s="1" t="s">
         <v>12</v>
@@ -1162,9 +1165,6 @@
       </c>
       <c r="H26" s="3" t="s">
         <v>13</v>
-      </c>
-      <c r="I26" s="1" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1172,10 +1172,10 @@
         <v>45</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="D27" s="1" t="s">
         <v>12</v>
@@ -1191,6 +1191,9 @@
       </c>
       <c r="H27" s="3" t="s">
         <v>13</v>
+      </c>
+      <c r="I27" s="1" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1198,7 +1201,7 @@
         <v>46</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C28" s="1" t="s">
         <v>11</v>
@@ -1220,14 +1223,30 @@
       </c>
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="4"/>
-      <c r="B29" s="4"/>
-      <c r="C29" s="4"/>
-      <c r="D29" s="4"/>
-      <c r="E29" s="4"/>
-      <c r="F29" s="4"/>
-      <c r="G29" s="4"/>
-      <c r="H29" s="4"/>
+      <c r="A29" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B29" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D29" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="E29" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F29" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="G29" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="H29" s="3" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="4"/>
@@ -1279,15 +1298,15 @@
       <c r="G34" s="4"/>
       <c r="H34" s="4"/>
     </row>
-    <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="4"/>
-      <c r="B38" s="4"/>
-      <c r="C38" s="4"/>
-      <c r="D38" s="4"/>
-      <c r="E38" s="4"/>
-      <c r="F38" s="4"/>
-      <c r="G38" s="4"/>
-      <c r="H38" s="4"/>
+    <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="4"/>
+      <c r="B35" s="4"/>
+      <c r="C35" s="4"/>
+      <c r="D35" s="4"/>
+      <c r="E35" s="4"/>
+      <c r="F35" s="4"/>
+      <c r="G35" s="4"/>
+      <c r="H35" s="4"/>
     </row>
     <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="4"/>
@@ -1299,13 +1318,23 @@
       <c r="G39" s="4"/>
       <c r="H39" s="4"/>
     </row>
+    <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="4"/>
+      <c r="B40" s="4"/>
+      <c r="C40" s="4"/>
+      <c r="D40" s="4"/>
+      <c r="E40" s="4"/>
+      <c r="F40" s="4"/>
+      <c r="G40" s="4"/>
+      <c r="H40" s="4"/>
+    </row>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="H2:H23 H25:H28" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="H2:H24 H26:H29" type="list">
       <formula1>"true,false"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="B2:B28" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="B2:B29" type="list">
       <formula1>"uint8_t,int8_t,uint16_t,int16_t,uint32_t,int32_t,float"</formula1>
       <formula2>0</formula2>
     </dataValidation>

</xml_diff>